<commit_message>
Update Google-Sheets-ready file to the 20 TikTok-confirmed creators
Replaces the previous mixed candidate set with the filtered list (25
minus the 5 without an actual TikTok citation), using text-rendered bar
charts instead of embedded chart objects since those don't survive
Google's xlsx->Sheets conversion. Adds a "Removed (non-TikTok)" tab for
transparency on what was excluded and why.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LRu2GdUFAXzVJjxasqRvd5
</commit_message>
<xml_diff>
--- a/nh_creator_scout/NH_TikTok_Scout_ForGoogleSheets.xlsx
+++ b/nh_creator_scout/NH_TikTok_Scout_ForGoogleSheets.xlsx
@@ -8,8 +8,9 @@
   </bookViews>
   <sheets>
     <sheet name="Creators" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Chart Data" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Top Picks" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Top Picks" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Chart" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Removed (non-TikTok)" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -39,6 +40,36 @@
       <color theme="10"/>
       <sz val="12"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <color rgb="002E7D32"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <color rgb="00C62828"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <color rgb="001565C0"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color theme="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color theme="10"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="3">
@@ -81,15 +112,37 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -167,287 +220,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Saudi TikTok Creators Found, by Niche</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Chart Data'!B1</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Chart Data'!$A$2:$A$4</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Chart Data'!$B$2:$B$4</f>
-            </numRef>
-          </val>
-        </ser>
-        <dLbls>
-          <showVal val="1"/>
-        </dLbls>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Niche</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Candidates</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="11"/>
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Disclosed TikTok Followers (thousands) — 7 of 20 candidates</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="bar"/>
-        <grouping val="clustered"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Chart Data'!B7</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Chart Data'!$A$8:$A$13</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Chart Data'!$B$8:$B$13</f>
-            </numRef>
-          </val>
-        </ser>
-        <dLbls>
-          <showVal val="1"/>
-        </dLbls>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Followers (K)</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Handle</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>4</col>
-      <colOff>0</colOff>
-      <row>1</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="5040000" cy="2880000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>4</col>
-      <colOff>0</colOff>
-      <row>19</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="5760000" cy="3600000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="2" name="Chart 2"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -742,11 +514,11 @@
   <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="42" customWidth="1" min="4" max="4"/>
-    <col width="39" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
     <col width="42" customWidth="1" min="6" max="6"/>
     <col width="42" customWidth="1" min="7" max="7"/>
     <col width="42" customWidth="1" min="8" max="8"/>
@@ -776,7 +548,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Followers (approx.)</t>
+          <t>Followers</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -796,7 +568,7 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Link Basis</t>
+          <t>Status</t>
         </is>
       </c>
     </row>
@@ -835,11 +607,7 @@
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Cited directly in research sources</t>
-        </is>
-      </c>
+      <c r="I2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -876,11 +644,7 @@
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Cited directly in research sources</t>
-        </is>
-      </c>
+      <c r="I3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -888,7 +652,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>ملاذ المصري / Malaz Al-Masri</t>
+          <t>Omar — "تجارة الكترونية بالعربي"</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -898,7 +662,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>@malazmarketing</t>
+          <t>@maketingomar</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -908,22 +672,18 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>E-commerce/digital marketing training, Salla &amp; Shopify store setup, TikTok/Meta ad campaigns</t>
+          <t>Arabic-language e-commerce content</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Deepest professional credentials of any e-commerce candidate found; long track record training Saudi merchants on Salla/Shopify</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Flag: nationality uncertain (possibly Egyptian, Saudi-market based)</t>
-        </is>
-      </c>
+          <t>Only verifiable TikTok presence found for this exact search angle</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Derived from verified handle (not independently re-clicked)</t>
+          <t>Insufficient verification — bare handle only</t>
         </is>
       </c>
     </row>
@@ -933,44 +693,40 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Ecommerce Academy / Katib School (أيت كاتب محمد)</t>
+          <t>د. اسعد رزق / Dr. Assad Rizq</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>E-commerce</t>
+          <t>Trading</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>@katibschool</t>
+          <t>@assadalsharef</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>n/a on TikTok</t>
+          <t>~1.1M (per search snippet)</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Free e-commerce training, "from A to Z"</t>
+          <t>Crypto/blockchain education (Bitcoin, altcoins), "how to build wealth with crypto"</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Established free e-commerce training brand</t>
+          <t>Unusually strong personal-credibility narrative (doctor-turned-crypto-educator), large following, Saudi hashtags (#السعودية)</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Flag: nationality likely non-Saudi (Moroccan naming pattern), not confirmed Saudi</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>Derived from verified handle (not independently re-clicked)</t>
-        </is>
-      </c>
+          <t>Crypto education content — verify no unlicensed investment-scheme promotion; "build wealth" framing leans aspirational-marketing</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -978,17 +734,17 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Omar — "تجارة الكترونية بالعربي"</t>
+          <t>بسام بن سليمان العبيد / Bassam bin Solaiman Al-Obaid</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>E-commerce</t>
+          <t>Trading</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>@maketingomar</t>
+          <t>@bin_solaiman</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -998,24 +754,20 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Arabic-language e-commerce content</t>
+          <t>US stock/options trading strategies, also covers Saudi market (#الاسهم_السعودية)</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Only verifiable TikTok presence found for this exact search angle</t>
+          <t>Strongest verifiable professional credential of the set (mainstream financial-press byline)</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Insufficient verification — bare handle only</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>Cited directly in research sources</t>
-        </is>
-      </c>
+          <t>Options-trading content carries inherent leverage/risk; no red flags found beyond that</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -1023,7 +775,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>فؤاد الحربي / Fuad Al-Harbi</t>
+          <t>محمد الباهلي / Muhammad Al-Bahli</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -1033,7 +785,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>@fuad8k</t>
+          <t>@m_albahly</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -1043,24 +795,20 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Saudi stock market (Tadawul) beginner education — explicitly no crypto, no fund management</t>
+          <t>Saudi stock market (Tadawul) news/education — dividend stocks, sukuk, automated "rebound zone" chart screens</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Explicit "stocks only, no crypto, no money management" positioning suggests deliberate compliance awareness</t>
+          <t>Consistently labels content "not a recommendation" (ليست توصية) across videos — better compliance hygiene than most</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Paid course sold via social media — verify he isn't implying licensed advisory status</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>Derived from verified handle (not independently re-clicked)</t>
-        </is>
-      </c>
+          <t>Automated "screening" videos could be read as stock tips despite disclaimers</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -1068,7 +816,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>تركي الحربي / Turki Al-Harbi</t>
+          <t>المستر سلطان المضحي / Mr. Sultan Al-Mudhi</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -1078,34 +826,30 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>@kii31t</t>
+          <t>@mrwallstreets.com</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>n/a on TikTok</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Personal investing/savings education; sells an "intelligent investment package" (261 SAR)</t>
+          <t>US stocks, options contracts, gold, oil, crypto — framed around Saudi CMA-approved trading platforms</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Cross-platform Saudi investment educator</t>
+          <t>Content directly addresses Saudi regulatory approval status of brokers — audience-relevant and somewhat compliance-aware</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Sells a paid "investment package" without disclosed licensing — potential unlicensed-advice risk</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>Derived from verified handle (not independently re-clicked)</t>
-        </is>
-      </c>
+          <t>Options/leveraged-instrument education for retail audience carries elevated risk profile even when not "hype" style</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -1113,7 +857,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>@deserttrader6906</t>
+          <t>العمدة أبو أحمد الاسهم / Al-Omda Abu Ahmad</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1123,32 +867,28 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>@deserttrader6906</t>
+          <t>@abo_ahmed_al3mda</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>~52K (per influencer-listing snippet)</t>
+          <t>~11.9K</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>US stock market + crypto (Bitcoin, altcoins), general investing</t>
+          <t>US stock technical analysis / "fractal equations"; explicitly "not investment recommendations"</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Bio explicitly states content is personal opinion, not financial advice — a compliance-conscious disclaimer</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>None major noted</t>
-        </is>
-      </c>
+          <t>Niche technical-analysis angle</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Derived from verified handle (not independently re-clicked)</t>
+          <t>Flag: Gulf-Arabic content, Saudi base unconfirmed (could be another Gulf state)</t>
         </is>
       </c>
     </row>
@@ -1158,42 +898,38 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>د. اسعد رزق / Dr. Assad Rizq</t>
+          <t>مطر الشمري / Matar Al-Shammari</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Trading</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>@assadalsharef</t>
+          <t>@mnfr60</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>~1.1M (per search snippet)</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Crypto/blockchain education (Bitcoin, altcoins), "how to build wealth with crypto"</t>
+          <t>Real-estate &amp; mortgage-financing advisory: refinancing vs. rescheduling, contract-signing tips, avoiding bad financing decisions</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Unusually strong personal-credibility narrative (doctor-turned-crypto-educator), large following, Saudi hashtags (#السعودية)</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>Crypto education content — verify no unlicensed investment-scheme promotion; "build wealth" framing leans aspirational-marketing</t>
-        </is>
-      </c>
+          <t>Clearest example of ongoing real-estate/financing education content by a self-identified Saudi consultant</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Derived from verified handle (not independently re-clicked)</t>
+          <t>Note: also surfaced independently in the earlier Northouse Finance scout (real-estate/تمويل عقاري angle) as @mnfr10 — same individual, cross-project convergence</t>
         </is>
       </c>
     </row>
@@ -1203,44 +939,36 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>بسام بن سليمان العبيد / Bassam bin Solaiman Al-Obaid</t>
+          <t>سعد الغامدي / Saad Al-Ghamdi</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Trading</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>@bin_solaiman</t>
+          <t>@jubail_aqari</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>~33.5K (165.9K likes)</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>US stock/options trading strategies, also covers Saudi market (#الاسهم_السعودية)</t>
+          <t>Local property marketing/listings for Jubail (Eastern Province); REGA-licensed ("معتمد من الهيئة العقارية" per bio/hashtags)</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Strongest verifiable professional credential of the set (mainstream financial-press byline)</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>Options-trading content carries inherent leverage/risk; no red flags found beyond that</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>Derived from verified handle (not independently re-clicked)</t>
-        </is>
-      </c>
+          <t>Named, licensed individual agent creator — precise match for "real-estate agent content"</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -1248,42 +976,38 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>محمد الباهلي / Muhammad Al-Bahli</t>
+          <t>عقار AQAR (Aqar App)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Trading</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>@m_albahly</t>
+          <t>@aqarapp</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>99.8K (362.7K likes)</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Saudi stock market (Tadawul) news/education — dividend stocks, sukuk, automated "rebound zone" chart screens</t>
+          <t>Saudi Arabia's largest real-estate listings/marketing platform (financing, leasing, market data)</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Consistently labels content "not a recommendation" (ليست توصية) across videos — better compliance hygiene than most</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>Automated "screening" videos could be read as stock tips despite disclaimers</t>
-        </is>
-      </c>
+          <t>Dominant brand in Saudi real-estate content — company/platform account, not an individual creator</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Derived from verified handle (not independently re-clicked)</t>
+          <t>Note: company/platform account, not an individual creator</t>
         </is>
       </c>
     </row>
@@ -1293,17 +1017,17 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>المستر سلطان المضحي / Mr. Sultan Al-Mudhi</t>
+          <t>عقارات الرياض / Riyadh Real Estate</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Trading</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>@mrwallstreets.com</t>
+          <t>@aqaar_1</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1313,22 +1037,18 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>US stocks, options contracts, gold, oil, crypto — framed around Saudi CMA-approved trading platforms</t>
+          <t>Riyadh-focused property listings/showcase content</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Content directly addresses Saudi regulatory approval status of brokers — audience-relevant and somewhat compliance-aware</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>Options/leveraged-instrument education for retail audience carries elevated risk profile even when not "hype" style</t>
-        </is>
-      </c>
+          <t>Plausible Riyadh listings account</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Derived from verified handle (not independently re-clicked)</t>
+          <t>Low confidence — no bio/credentials verifiable</t>
         </is>
       </c>
     </row>
@@ -1338,44 +1058,36 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>العمدة أبو أحمد الاسهم / Al-Omda Abu Ahmad</t>
+          <t>شقق ايجار يومي الملقا الرياض</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Trading</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>@abo_ahmed_al3mda</t>
+          <t>@rr05l</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>~11.9K</t>
+          <t>~37K (1.5M likes)</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>US stock technical analysis / "fractal equations"; explicitly "not investment recommendations"</t>
+          <t>Daily/short-term rental apartment listings in Al-Malqa and central/north Riyadh</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Niche technical-analysis angle</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>Flag: Gulf-Arabic content, Saudi base unconfirmed (could be another Gulf state)</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>Derived from verified handle (not independently re-clicked)</t>
-        </is>
-      </c>
+          <t>Real-estate/rental-listing niche, closer to classifieds than education</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -1383,7 +1095,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>مطر الشمري / Matar Al-Shammari</t>
+          <t>عقار وأكثر / Aqar wa Akthar</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1393,7 +1105,7 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>@mnfr60</t>
+          <t>@aqari_jdh</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1403,22 +1115,18 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Real-estate &amp; mortgage-financing advisory: refinancing vs. rescheduling, contract-signing tips, avoiding bad financing decisions</t>
+          <t>Handle name suggests Jeddah-area real estate ("jdh"); specific content niche not independently confirmed</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Clearest example of ongoing real-estate/financing education content by a self-identified Saudi consultant</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>Note: also surfaced independently in the earlier Northouse Finance scout (real-estate/تمويل عقاري angle) as @mnfr10 — same individual, cross-project convergence</t>
-        </is>
-      </c>
+          <t>Lead for further vetting only</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr"/>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>Cited directly in research sources</t>
+          <t>Low confidence — unverified beyond handle existing</t>
         </is>
       </c>
     </row>
@@ -1428,7 +1136,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>سعد الغامدي / Saad Al-Ghamdi</t>
+          <t>عقار المملكة / Kingdom Real Estate (cluster)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1438,28 +1146,28 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>@jubail_aqari</t>
+          <t>@kingdom_aqar (related: @kingdomaqar, @aqar_ksa__)</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>~33.5K (165.9K likes)</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Local property marketing/listings for Jubail (Eastern Province); REGA-licensed ("معتمد من الهيئة العقارية" per bio/hashtags)</t>
+          <t>Saudi real-estate/development news (e.g. Riyadh infrastructure/road-project coverage tied to property value)</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Named, licensed individual agent creator — precise match for "real-estate agent content"</t>
+          <t>Real-estate news/commentary niche</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr"/>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Cited directly in research sources</t>
+          <t>Low confidence — handle cluster needs manual disambiguation</t>
         </is>
       </c>
     </row>
@@ -1469,44 +1177,36 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>عقار AQAR (Aqar App)</t>
+          <t>رعد الحربي (أبو دانه) / Raad Al-Harbi ("Abu Danah")</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Trading</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>@aqarapp</t>
+          <t>@abu_danah00</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>99.8K (362.7K likes)</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Saudi Arabia's largest real-estate listings/marketing platform (financing, leasing, market data)</t>
+          <t>Saudi (Tadawul) stock and fund trading education — technical/fundamental analysis, portfolio building, beginner-to-pro courses</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Dominant brand in Saudi real-estate content — company/platform account, not an individual creator</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>Note: company/platform account, not an individual creator</t>
-        </is>
-      </c>
-      <c r="I17" s="2" t="inlineStr">
-        <is>
-          <t>Cited directly in research sources</t>
-        </is>
-      </c>
+          <t>Named individual (tribal surname Al-Harbi) with self-declared Saudi flag; cross-verified via 3 independent properties beyond the TikTok page (X, YouTube, own academy site); risk-aware framing, not signal-selling</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr"/>
+      <c r="I17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1514,44 +1214,36 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>عقارات الرياض / Riyadh Real Estate</t>
+          <t>محمد الخضير / Mohammed Alkhudhair</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Trading</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>@aqaar_1</t>
+          <t>@mohakhuu</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>~114K</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Riyadh-focused property listings/showcase content</t>
+          <t>Retail investing/fintech education — comparing Saudi investment/trading apps (Derayah, Tamra, Malaa, Drahim, Abyan, Al Rajhi Capital), tracking Tadawul holdings</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Plausible Riyadh listings account</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>Low confidence — no bio/credentials verifiable</t>
-        </is>
-      </c>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>Cited directly in research sources</t>
-        </is>
-      </c>
+          <t>Named individual with a disclosed, non-hype comparison methodology; strongly Saudi-contextualized content (PIF, Saudia Airlines, Saudi banks, CMA-licensed apps); cross-verified via X + Instagram under consistent name/photo</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -1559,7 +1251,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>شقق ايجار يومي الملقا الرياض</t>
+          <t>عماد منشي / Emad Munshi</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -1569,30 +1261,26 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>@rr05l</t>
+          <t>@emad_munshi</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>~37K (1.5M likes)</t>
+          <t>~165.7K (543.3K likes)</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Daily/short-term rental apartment listings in Al-Malqa and central/north Riyadh</t>
+          <t>Real-estate investment consultancy/analysis (Jeddah apartment/land investing, market-timing videos)</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Real-estate/rental-listing niche, closer to classifieds than education</t>
+          <t>Named individual with a consistent identity across TikTok/X/Instagram/Snapchat/website; explicit Jeddah, Saudi tie via his company, independently confirmed beyond the TikTok page</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr"/>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>Cited directly in research sources</t>
-        </is>
-      </c>
+      <c r="I19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -1600,7 +1288,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>عقار وأكثر / Aqar wa Akthar</t>
+          <t>سعد بن محمد التويم / Saad bin Mohammed Al-Tuwaim</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1610,34 +1298,26 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>@aqari_jdh</t>
+          <t>@saadaltwaim1</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>~133.2K (490.1K likes)</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Handle name suggests Jeddah-area real estate ("jdh"); specific content niche not independently confirmed</t>
+          <t>Real-estate market commentary, appraisal/valuation education, Riyadh market analysis (demand trends, pricing)</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Lead for further vetting only</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t>Low confidence — unverified beyond handle existing</t>
-        </is>
-      </c>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>Cited directly in research sources</t>
-        </is>
-      </c>
+          <t>Real named individual with a documented corporate role (Tathmen chairman), independently confirmed via the company's own site and 4 distinct platforms (X, YouTube, Facebook, LinkedIn) under a consistent name</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -1645,7 +1325,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>عقار المملكة / Kingdom Real Estate (cluster)</t>
+          <t>طارق شقرون / Tariq Shagroon ("Mr. Broker")</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -1655,34 +1335,26 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>@kingdom_aqar (related: @kingdomaqar, @aqar_ksa__)</t>
+          <t>@tshagroon</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>~194.8K</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Saudi real-estate/development news (e.g. Riyadh infrastructure/road-project coverage tied to property value)</t>
+          <t>Personal real-estate consulting/brokerage content in Madinah — property tours, buy/sell/invest Q&amp;A</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Real-estate news/commentary niche</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>Low confidence — handle cluster needs manual disambiguation</t>
-        </is>
-      </c>
-      <c r="I21" s="2" t="inlineStr">
-        <is>
-          <t>Cited directly in research sources</t>
-        </is>
-      </c>
+          <t>Named individual (not a brand/listings account); explicit Madinah tie across content and company; independently corroborated by two separate news/feature articles plus a distinct company website</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr"/>
+      <c r="I21" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1717,11 +1389,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1732,126 +1405,145 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Candidates</t>
+          <t>TikTok Account (click)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Rank Note</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>E-commerce</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>5</v>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>@econabdallah</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>#1 — only e-commerce candidate with fully cross-verified Saudi nationality (Riyadh), ~178K TikTok followers, content squarely in dropshipping/store-launch niche across every platform</t>
+        </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>@adeel8866</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>#2 — strong niche fit (dropshipping suppliers, sourcing, tutorials) with explicit Saudi-market hashtagging, though personal nationality confirmation is thinner</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Trading</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>@assadalsharef</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>#1 — leads on reach (~1.1M) and a distinctive doctor-turned-crypto-educator credibility narrative, though "build wealth with crypto" framing warrants compliance scrutiny</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Trading</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>@bin_solaiman</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>#2 — most professionally credentialed (financial-press byline, market-data consultancy) with genuine Saudi-market hashtag activity</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5"/>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>Handle</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
-        <is>
-          <t>Followers (thousands)</t>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>@mnfr60</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>#1 — most clearly documented individual creator, consistently branded across TikTok/X/Snapchat/YouTube as a real-estate and mortgage-financing consultant with a repeatable content format</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>@econabdallah</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>178.1</v>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Real Estate</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>@jubail_aqari</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>#2 — named, REGA-credentialed local property marketer with a concrete follower count (33.5K) and a clear regional niche (Jubail/Eastern Province)</t>
+        </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>@deserttrader6906</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>@assadalsharef</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>1100</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>@abo_ahmed_al3mda</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>11.9</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>@jubail_aqari</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>33.5</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Real Estate</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>@aqarapp</t>
         </is>
       </c>
-      <c r="B12" t="n">
-        <v>99.8</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>@rr05l</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>37</v>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>#3 — not an individual, but the single best-verified, largest real-estate brand active on Saudi TikTok (99.8K followers), backed by independent press coverage</t>
+        </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId7"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1861,196 +1553,537 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Candidates by Niche (20 TikTok-confirmed)</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="n"/>
+      <c r="C1" s="5" t="n"/>
+      <c r="D1" s="5" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="n"/>
+      <c r="B2" s="5" t="n"/>
+      <c r="C2" s="5" t="n"/>
+      <c r="D2" s="5" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Niche</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>TikTok Account (click)</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Rank Note</t>
-        </is>
-      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>Bar</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>E-commerce</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>█████████</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Trading</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>█████████████████████</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Real Estate</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>██████████████████████████████</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Disclosed TikTok Followers (thousands)</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n"/>
+      <c r="C7" s="5" t="n"/>
+      <c r="D7" s="5" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="n"/>
+      <c r="B8" s="5" t="n"/>
+      <c r="C8" s="5" t="n"/>
+      <c r="D8" s="5" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Handle</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Niche</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="inlineStr">
+        <is>
+          <t>Followers (K)</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Bar</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>@assadalsharef</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Trading</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>1100</v>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>████████████████████████████████████████</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>@tshagroon</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Real Estate</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>194.8</v>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>███████</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>@econabdallah</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>E-commerce</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>178.1</v>
+      </c>
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>██████</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>@emad_munshi</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Real Estate</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>165.7</v>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>██████</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>@saadaltwaim1</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Real Estate</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>133.2</v>
+      </c>
+      <c r="D14" s="12" t="inlineStr">
+        <is>
+          <t>█████</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>@mohakhuu</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Trading</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>114</v>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>████</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>@aqarapp</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Real Estate</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>99.8</v>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>████</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>@rr05l</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Real Estate</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>█</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>@jubail_aqari</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Real Estate</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>33.5</v>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>█</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>@abo_ahmed_al3mda</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Trading</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>█</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="55" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="39" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Removed from the original 25 — sourced from non-TikTok evidence only</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="n"/>
+      <c r="C1" s="5" t="n"/>
+      <c r="D1" s="5" t="n"/>
+      <c r="E1" s="5" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="5" t="n"/>
+      <c r="B2" s="5" t="n"/>
+      <c r="C2" s="5" t="n"/>
+      <c r="D2" s="5" t="n"/>
+      <c r="E2" s="5" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>Name (AR/EN)</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Niche</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Handle</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>Followers</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Why removed (source basis)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>ملاذ المصري / Malaz Al-Masri</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>E-commerce</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>@econabdallah</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>#1 — only e-commerce candidate with fully cross-verified Saudi nationality (Riyadh), ~178K TikTok followers, content squarely in dropshipping/store-launch niche across every platform</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>@malazmarketing</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>https://malazmarketing.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Ecommerce Academy / Katib School (أيت كاتب محمد)</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>E-commerce</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>@adeel8866</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>#2 — strong niche fit (dropshipping suppliers, sourcing, tutorials) with explicit Saudi-market hashtagging, though personal nationality confirmation is thinner</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>E-commerce</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>@malazmarketing</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>#3 — deepest professional credentials of any e-commerce candidate, but flagged: likely-Egyptian background means Saudi nationality (vs. market residency) is unconfirmed</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>@katibschool</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>n/a on TikTok</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/katibschool/ ; https://katibschool.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>فؤاد الحربي / Fuad Al-Harbi</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Trading</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>@assadalsharef</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>#1 — leads on reach (~1.1M) and a distinctive doctor-turned-crypto-educator credibility narrative, though "build wealth with crypto" framing warrants compliance scrutiny</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>@fuad8k</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>https://fuadacademy.com ; https://x.com/fuad7333</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>تركي الحربي / Turki Al-Harbi</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Trading</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>@bin_solaiman</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>#2 — most professionally credentialed (financial-press byline, market-data consultancy) with genuine Saudi-market hashtag activity</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>@kii31t</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>n/a on TikTok</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>Search snippets for "kii31t تركي الحربي"; Snapchat profile page</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>@deserttrader6906</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Trading</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>@fuad8k</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>#3 — cleanest self-imposed compliance boundary of the group: stocks-only education, explicitly no crypto or fund management</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Real Estate</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>@mnfr60</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>#1 — most clearly documented individual creator, consistently branded across TikTok/X/Snapchat/YouTube as a real-estate and mortgage-financing consultant with a repeatable content format</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Real Estate</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>@jubail_aqari</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>#2 — named, REGA-credentialed local property marketer with a concrete follower count (33.5K) and a clear regional niche (Jubail/Eastern Province)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Real Estate</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>@aqarapp</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>#3 — not an individual, but the single best-verified, largest real-estate brand active on Saudi TikTok (99.8K followers), backed by independent press coverage</t>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>@deserttrader6906</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>~52K (per influencer-listing snippet)</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Heepsy/aggregator listing describing account as "based in Saudi Arabia"</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId9"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>